<commit_message>
Promote Plus Code capture
</commit_message>
<xml_diff>
--- a/app/src/main/java/com/example/methodmesh/modules/pluscodecapture/docs/example_odk_plus_code.capture.xlsx
+++ b/app/src/main/java/com/example/methodmesh/modules/pluscodecapture/docs/example_odk_plus_code.capture.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -631,7 +631,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>com.example.methodmesh.EXECUTE_METHOD(method_id='plus_code.capture',input_code_length=${code_length_input},input_gps_average_seconds=${gps_average_seconds_input},input_basemap_mode=${basemap_mode_input},input_grid_span_cells=${grid_span_cells_input},return_mode='flat')</t>
+          <t>com.example.methodmesh.EXECUTE_METHOD(method_id='plus_code.capture',input_code_length=${code_length_input},input_gps_average_seconds=${gps_average_seconds_input},input_basemap_mode=${basemap_mode_input},input_grid_span_cells=${grid_span_cells_input},input_payload_mode='FULL',return_mode='flat')</t>
         </is>
       </c>
     </row>
@@ -643,17 +643,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>plus_code</t>
+          <t>methodmesh_execution_id</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Selected full Plus Code</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>MethodMesh execution ID</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -665,17 +660,17 @@
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>plus_code_centroid_latitude</t>
+          <t>methodmesh_status</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Selected cell centroid latitude</t>
+          <t>MethodMesh status</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -687,17 +682,22 @@
     <row r="9" ht="15" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>plus_code_centroid_longitude</t>
+          <t>plus_code</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Selected cell centroid longitude</t>
+          <t>Selected full Plus Code</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -709,17 +709,17 @@
     <row r="10" ht="15" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>plus_code_gps_latitude</t>
+          <t>methodmesh_full_json</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Original GPS latitude</t>
+          <t>MethodMesh metadata JSON</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -731,318 +731,67 @@
     <row r="11" ht="15" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>plus_code_gps_longitude</t>
+          <t>selected_summary</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Original GPS longitude</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Selected location: ${plus_code}</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>${plus_code} != ''</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>plus_code_gps_accuracy_m</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>GPS accuracy (m)</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>plus_code_capture_end</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>plus_code_gps_fix_count</t>
+          <t>plus_code_done</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GPS fix count</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>plus_code_selected_time_iso</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Selected time</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>plus_code_status</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MethodMesh status</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>plus_code_length</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Plus Code length</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>plus_code_basemap_mode</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Requested basemap mode</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>plus_code_basemap_actual_source</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Actual basemap source</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>plus_code_error</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Capture error</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>plus_code_audit_json</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Audit JSON</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>selected_summary</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Selected location: ${plus_code}</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+          <t>Plus Code captured: ${plus_code}</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>${plus_code} != ''</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>gps_summary</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>GPS: ${plus_code_gps_latitude}, ${plus_code_gps_longitude}; accuracy ±${plus_code_gps_accuracy_m} m</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>${plus_code_gps_latitude} != ''</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>audit_note</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Audit JSON is captured in the hidden field for export/audit.</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>false()</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>end_group</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>plus_code_done</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Plus Code captured: ${plus_code}</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>${plus_code} != ''</t>
-        </is>
-      </c>
-    </row>
+    <row r="14" ht="15" customHeight="1"/>
+    <row r="15" ht="15" customHeight="1"/>
+    <row r="16" ht="15" customHeight="1"/>
+    <row r="17" ht="15" customHeight="1"/>
+    <row r="18" ht="15" customHeight="1"/>
+    <row r="19" ht="15" customHeight="1"/>
+    <row r="20" ht="15" customHeight="1"/>
+    <row r="21" ht="15" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1054,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.440000057220459" customWidth="1" min="1" max="1"/>
@@ -1177,7 +926,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Online maps with fallback</t>
+          <t>Street map</t>
         </is>
       </c>
     </row>
@@ -1206,29 +955,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>street</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Street map</t>
+          <t>Grid only</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>basemap_mode</t>
+          <t>grid_span_cells</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>grid</t>
+          <t>129</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Grid only</t>
+          <t>Wide overview</t>
         </is>
       </c>
     </row>
@@ -1240,12 +989,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wide overview</t>
+          <t>Field</t>
         </is>
       </c>
     </row>
@@ -1257,46 +1006,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>grid_span_cells</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
           <t>Close</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>grid_span_cells</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Very close</t>
         </is>
       </c>
     </row>

</xml_diff>